<commit_message>
Convert excel to Json and modify sayID
</commit_message>
<xml_diff>
--- a/Data/DataDemo.xlsx
+++ b/Data/DataDemo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EJL\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unity\EmotionCrista\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF3E361-98D8-4887-B20C-C2538A0D4FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BF6287-0E5C-4CFD-A5EC-9A02FB09A767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{E729D64F-B358-4F37-A2EC-6B22D44EC8E5}"/>
+    <workbookView xWindow="29190" yWindow="-4845" windowWidth="15720" windowHeight="13740" xr2:uid="{E729D64F-B358-4F37-A2EC-6B22D44EC8E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Rule" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -289,6 +289,14 @@
   </si>
   <si>
     <t>위에 SpriteName을 적었을 때 필수</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cmd 창 명령어: python &lt;__.py&gt; &lt;__.xlsx&gt; &lt;sheetname&gt; &lt;__.json&gt;</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"Missing optional dependency" 오류 뜨면: pip install -r Requirements.txt</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -383,13 +391,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -698,7 +706,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -706,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCC34366-1101-4A18-8B57-8FFEE31C0A44}">
-  <dimension ref="B1:E44"/>
+  <dimension ref="B1:E45"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16.5" style="3" customWidth="1"/>
@@ -716,268 +724,275 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
+      <c r="B1" s="3" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="1"/>
+      <c r="B2" s="3" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="5" t="s">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="5"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-    </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6" t="s">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="5" t="s">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="5"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="5"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="5" t="s">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>39</v>
-      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" s="1"/>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="1"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="1"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="C31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C33" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C34" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C37" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C38" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="39" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C43" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C44" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C45" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>